<commit_message>
chore: add seed production state and update expense report
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/reports/gastos-dev-infra-nov2025-feb2026.xlsx
+++ b/docs/reports/gastos-dev-infra-nov2025-feb2026.xlsx
@@ -1,42 +1,93 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\kris\ceibatic\products\alquemist\docs\reports\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DB32F5-575A-44D9-A7CB-F8B4C116C7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="26640" windowHeight="14370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Gastos Dev-Infra" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+  <si>
+    <t>Alquemist — Reporte de Gastos Dev/Infra</t>
+  </si>
+  <si>
+    <t>Período: Noviembre 2025 - Febrero 2026</t>
+  </si>
+  <si>
+    <t>Moneda: USD</t>
+  </si>
+  <si>
+    <t>Servicio</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Vercel Pro (1 plan)</t>
+  </si>
+  <si>
+    <t>Claude Max (1 cuenta)</t>
+  </si>
+  <si>
+    <t>Google Workspace Starter (1 agrodinamic)</t>
+  </si>
+  <si>
+    <t>Google Workspace Starter (1 alquemist)</t>
+  </si>
+  <si>
+    <t>Maria Camila (16.6%)</t>
+  </si>
+  <si>
+    <t>Ernesto  (16.6%)</t>
+  </si>
+  <si>
+    <t>David  (16.6%)</t>
+  </si>
+  <si>
+    <t>Cristian  (50%)</t>
+  </si>
+  <si>
+    <t>TOTAL COMPARTIDO</t>
+  </si>
+  <si>
+    <t>TOTAL AGRODINAMIC</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="2">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="60" formatCode="$#,##0.00"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -45,12 +96,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -65,15 +128,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="10">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -398,55 +479,71 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="38.875" customWidth="1"/>
+    <col min="2" max="6" width="12.875" customWidth="1"/>
+    <col min="8" max="8" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Alquemist — Reporte de Gastos Dev/Infra</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Período: Noviembre 2025 - Febrero 2026</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>Moneda: USD</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Servicio</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Nov 2025</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Dic 2025</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Ene 2026</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Feb 2026</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Total</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Google Workspace Starter (1 cuenta)</v>
+    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3">
+        <v>45962</v>
+      </c>
+      <c r="C5" s="3">
+        <v>45992</v>
+      </c>
+      <c r="D5" s="3">
+        <v>45658</v>
+      </c>
+      <c r="E5" s="3">
+        <v>45689</v>
+      </c>
+      <c r="F5" s="3">
+        <v>46082</v>
+      </c>
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>7</v>
       </c>
       <c r="B6" s="1">
         <v>7.2</v>
@@ -461,77 +558,250 @@
         <v>7.2</v>
       </c>
       <c r="F6" s="1">
-        <v>28.8</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Claude Pro (1 cuenta)</v>
-      </c>
-      <c r="B7" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G6" s="1">
+        <f>SUM(B6:F6)</f>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="F7" s="1">
+        <v>7.2</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" ref="G7:G17" si="0">SUM(B7:F7)</f>
+        <v>14.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="1">
+        <v>50</v>
+      </c>
+      <c r="C8" s="1">
+        <v>50</v>
+      </c>
+      <c r="D8" s="1">
+        <v>50</v>
+      </c>
+      <c r="E8" s="1">
+        <v>50</v>
+      </c>
+      <c r="F8" s="1">
+        <v>50</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1">
         <v>20</v>
       </c>
-      <c r="C7" s="1">
+      <c r="F9" s="1">
         <v>20</v>
       </c>
-      <c r="D7" s="1">
-        <v>20</v>
-      </c>
-      <c r="E7" s="1">
-        <v>20</v>
-      </c>
-      <c r="F7" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Vercel Pro (1 plan)</v>
-      </c>
-      <c r="B8" s="1">
-        <v>20</v>
-      </c>
-      <c r="C8" s="1">
-        <v>20</v>
-      </c>
-      <c r="D8" s="1">
-        <v>20</v>
-      </c>
-      <c r="E8" s="1">
-        <v>20</v>
-      </c>
-      <c r="F8" s="1">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>TOTAL MENSUAL</v>
-      </c>
-      <c r="B10">
-        <v>47.2</v>
-      </c>
-      <c r="C10">
-        <v>47.2</v>
-      </c>
-      <c r="D10">
-        <v>47.2</v>
-      </c>
-      <c r="E10">
-        <v>47.2</v>
-      </c>
-      <c r="F10">
-        <v>188.8</v>
-      </c>
-    </row>
+      <c r="G9" s="1">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G10" s="1"/>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="9">
+        <f>SUM(B7:B10)</f>
+        <v>50</v>
+      </c>
+      <c r="C11" s="9">
+        <f>SUM(C7:C10)</f>
+        <v>50</v>
+      </c>
+      <c r="D11" s="9">
+        <f>SUM(D7:D10)</f>
+        <v>50</v>
+      </c>
+      <c r="E11" s="9">
+        <f>SUM(E7:E10)</f>
+        <v>77.2</v>
+      </c>
+      <c r="F11" s="9">
+        <f>SUM(F7:F10)</f>
+        <v>77.2</v>
+      </c>
+      <c r="G11" s="9">
+        <f t="shared" si="0"/>
+        <v>304.39999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="7">
+        <f>B6</f>
+        <v>7.2</v>
+      </c>
+      <c r="C12" s="7">
+        <f>C6</f>
+        <v>7.2</v>
+      </c>
+      <c r="D12" s="7">
+        <f>D6</f>
+        <v>7.2</v>
+      </c>
+      <c r="E12" s="7">
+        <f>E6</f>
+        <v>7.2</v>
+      </c>
+      <c r="F12" s="7">
+        <f>F6</f>
+        <v>7.2</v>
+      </c>
+      <c r="G12" s="7">
+        <f t="shared" si="0"/>
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="5">
+        <f>B$11*(0.5/3)</f>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="C14" s="5">
+        <f>C$11*(0.5/3)</f>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="D14" s="5">
+        <f t="shared" ref="D14:F16" si="1">D$11*(0.5/3)</f>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="E14" s="5">
+        <f t="shared" si="1"/>
+        <v>12.866666666666667</v>
+      </c>
+      <c r="F14" s="5"/>
+      <c r="G14" s="7">
+        <f t="shared" si="0"/>
+        <v>37.86666666666666</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="5">
+        <f t="shared" ref="B15:C16" si="2">B$11*(0.5/3)</f>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="C15" s="5">
+        <f t="shared" si="2"/>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="D15" s="5">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="E15" s="5">
+        <f t="shared" si="1"/>
+        <v>12.866666666666667</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="7">
+        <f t="shared" si="0"/>
+        <v>37.86666666666666</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="5">
+        <f t="shared" si="2"/>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="C16" s="5">
+        <f t="shared" si="2"/>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="D16" s="5">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333321</v>
+      </c>
+      <c r="E16" s="5">
+        <f t="shared" si="1"/>
+        <v>12.866666666666667</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="7">
+        <f t="shared" si="0"/>
+        <v>37.86666666666666</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17" s="5">
+        <f>B$11*(0.5)</f>
+        <v>25</v>
+      </c>
+      <c r="C17" s="5">
+        <f t="shared" ref="C17:F17" si="3">C$11*(0.5)</f>
+        <v>25</v>
+      </c>
+      <c r="D17" s="5">
+        <f t="shared" si="3"/>
+        <v>25</v>
+      </c>
+      <c r="E17" s="5">
+        <f t="shared" si="3"/>
+        <v>38.6</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="7">
+        <f t="shared" si="0"/>
+        <v>113.6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
   </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F10"/>
+    <ignoredError sqref="A1:F4 A10:E10 B6:E6 A5 A9 E9" numberStoredAsText="1"/>
+    <ignoredError sqref="B11:F11" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>